<commit_message>
Add Unallocated Fee column to Forecast Amount variant
On the direct forecast-amount workbook, engagement managers type amounts that
may not sum to the fee, so the Dashboard by-engagement table gains an
Unallocated Fee (£) = total fee - total forecast entered. Coloured amber when
fee is still to spread, red when over-forecast, blank when fully forecast.
Only the Forecast Amount variant is affected. Formulas verified (zero errors),
cached values refreshed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHLa9TiLWycdAtWPCqjTQM
</commit_message>
<xml_diff>
--- a/Income_Forecast_ForecastAmount.xlsx
+++ b/Income_Forecast_ForecastAmount.xlsx
@@ -951,10 +951,10 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1">
+    <row r="23" ht="60" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>· Forecast and all amounts are GBP.   · Dates are the first of the month (shown as Sep-2026).   · Demo engagements M-1001/1002/1003 are examples — delete them once you add your own.</t>
+          <t>· Forecast and all amounts are GBP.   · The Dashboard's Unallocated Fee (£) column = total fee minus the forecast you've entered: amber = fee still to spread, red = over-forecast, blank = fully forecast.   · Dates are the first of the month (shown as Sep-2026).   · Demo engagements M-1001/1002/1003 are examples — delete them once you add your own.</t>
         </is>
       </c>
     </row>
@@ -4924,7 +4924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -4941,6 +4941,7 @@
     <col width="16" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5023,6 +5024,11 @@
           <t>Open Var (#)</t>
         </is>
       </c>
+      <c r="O4" s="5" t="inlineStr">
+        <is>
+          <t>Unallocated Fee (£)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="22" t="n">
@@ -5076,6 +5082,10 @@
         <f>IF($F5="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F5,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v>2</v>
       </c>
+      <c r="O5" s="17">
+        <f>IF($F5="","",I5-J5)</f>
+        <v>66000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="22" t="n">
@@ -5129,6 +5139,10 @@
         <f>IF($F6="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F6,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v>0</v>
       </c>
+      <c r="O6" s="17">
+        <f>IF($F6="","",I6-J6)</f>
+        <v>63000</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="22" t="n">
@@ -5182,6 +5196,10 @@
         <f>IF($F7="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F7,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v>0</v>
       </c>
+      <c r="O7" s="17">
+        <f>IF($F7="","",I7-J7)</f>
+        <v>21000</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="22" t="n">
@@ -5235,6 +5253,10 @@
         <f>IF($F8="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F8,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O8" s="17" t="str">
+        <f>IF($F8="","",I8-J8)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="22" t="n">
@@ -5288,6 +5310,10 @@
         <f>IF($F9="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F9,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O9" s="17" t="str">
+        <f>IF($F9="","",I9-J9)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="22" t="n">
@@ -5341,6 +5367,10 @@
         <f>IF($F10="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F10,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O10" s="17" t="str">
+        <f>IF($F10="","",I10-J10)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="22" t="n">
@@ -5394,6 +5424,10 @@
         <f>IF($F11="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F11,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O11" s="17" t="str">
+        <f>IF($F11="","",I11-J11)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="22" t="n">
@@ -5447,6 +5481,10 @@
         <f>IF($F12="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F12,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O12" s="17" t="str">
+        <f>IF($F12="","",I12-J12)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="22" t="n">
@@ -5500,6 +5538,10 @@
         <f>IF($F13="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F13,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O13" s="17" t="str">
+        <f>IF($F13="","",I13-J13)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="22" t="n">
@@ -5553,6 +5595,10 @@
         <f>IF($F14="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F14,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O14" s="17" t="str">
+        <f>IF($F14="","",I14-J14)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="22" t="n">
@@ -5606,6 +5652,10 @@
         <f>IF($F15="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F15,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O15" s="17" t="str">
+        <f>IF($F15="","",I15-J15)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="22" t="n">
@@ -5659,6 +5709,10 @@
         <f>IF($F16="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F16,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O16" s="17" t="str">
+        <f>IF($F16="","",I16-J16)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="27" t="inlineStr">
@@ -5714,6 +5768,10 @@
         <f>IF($F17="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F17,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O17" s="17" t="str">
+        <f>IF($F17="","",I17-J17)</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="F18" s="23" t="str">
@@ -5752,6 +5810,10 @@
         <f>IF($F18="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F18,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O18" s="17" t="str">
+        <f>IF($F18="","",I18-J18)</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="29" t="inlineStr">
@@ -5793,6 +5855,10 @@
       </c>
       <c r="N19" s="26" t="str">
         <f>IF($F19="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F19,'Forecast Log'!$P$5:$P$64,"YES"))</f>
+        <v/>
+      </c>
+      <c r="O19" s="17" t="str">
+        <f>IF($F19="","",I19-J19)</f>
         <v/>
       </c>
     </row>
@@ -5842,6 +5908,10 @@
         <f>IF($F20="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F20,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O20" s="17" t="str">
+        <f>IF($F20="","",I20-J20)</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="30" t="inlineStr">
@@ -5889,6 +5959,10 @@
         <f>IF($F21="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F21,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O21" s="17" t="str">
+        <f>IF($F21="","",I21-J21)</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="30" t="inlineStr">
@@ -5936,6 +6010,10 @@
         <f>IF($F22="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F22,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O22" s="17" t="str">
+        <f>IF($F22="","",I22-J22)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="F23" s="23" t="str">
@@ -5974,6 +6052,10 @@
         <f>IF($F23="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F23,'Forecast Log'!$P$5:$P$64,"YES"))</f>
         <v/>
       </c>
+      <c r="O23" s="17" t="str">
+        <f>IF($F23="","",I23-J23)</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="F24" s="23" t="str">
@@ -6010,6 +6092,10 @@
       </c>
       <c r="N24" s="26" t="str">
         <f>IF($F24="","",COUNTIFS('Forecast Log'!$A$5:$A$64,$F24,'Forecast Log'!$P$5:$P$64,"YES"))</f>
+        <v/>
+      </c>
+      <c r="O24" s="17" t="str">
+        <f>IF($F24="","",I24-J24)</f>
         <v/>
       </c>
     </row>
@@ -6094,13 +6180,21 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="O5:O24">
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="I28:I29">
-    <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="6" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B20">
-    <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="0">
+    <cfRule type="cellIs" priority="7" operator="greaterThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Reconcile Unallocated Fee against actuals for closed months
Fixes double-counting when a variance is reforecast into a later month. The
Unallocated Fee column now = Remaining Fee - forecast on months that don't yet
have an actual (SUMPRODUCT over open months). Months already actualised are
counted at their actual, so the original forecast row stays untouched and
re-spreading a variance across future months reconciles Unallocated back to
zero. Forecast Amount variant only. Verified: reconciliation returns 0 after a
reforecast; zero formula errors; cached values refreshed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHLa9TiLWycdAtWPCqjTQM
</commit_message>
<xml_diff>
--- a/Income_Forecast_ForecastAmount.xlsx
+++ b/Income_Forecast_ForecastAmount.xlsx
@@ -951,10 +951,10 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="90" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>· Forecast and all amounts are GBP.   · The Dashboard's Unallocated Fee (£) column = total fee minus the forecast you've entered: amber = fee still to spread, red = over-forecast, blank = fully forecast.   · Dates are the first of the month (shown as Sep-2026).   · Demo engagements M-1001/1002/1003 are examples — delete them once you add your own.</t>
+          <t>· Forecast and all amounts are GBP.   · The Dashboard's Unallocated Fee (£) = fee not yet covered by actuals or by forecast on months still open. Months that already have an actual are counted at their actual, so the original forecast row stays untouched and re-spreading a variance across future months reconciles back to zero: amber = fee still to spread, red = over-forecast, blank = fully forecast.   · Dates are the first of the month (shown as Sep-2026).   · Demo engagements M-1001/1002/1003 are examples — delete them once you add your own.</t>
         </is>
       </c>
     </row>
@@ -5083,8 +5083,8 @@
         <v>2</v>
       </c>
       <c r="O5" s="17">
-        <f>IF($F5="","",I5-J5)</f>
-        <v>66000</v>
+        <f>IF($F5="","",L5-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F5)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
+        <v>67000</v>
       </c>
     </row>
     <row r="6">
@@ -5140,7 +5140,7 @@
         <v>0</v>
       </c>
       <c r="O6" s="17">
-        <f>IF($F6="","",I6-J6)</f>
+        <f>IF($F6="","",L6-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F6)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v>63000</v>
       </c>
     </row>
@@ -5197,8 +5197,8 @@
         <v>0</v>
       </c>
       <c r="O7" s="17">
-        <f>IF($F7="","",I7-J7)</f>
-        <v>21000</v>
+        <f>IF($F7="","",L7-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F7)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
+        <v>22000</v>
       </c>
     </row>
     <row r="8">
@@ -5254,7 +5254,7 @@
         <v/>
       </c>
       <c r="O8" s="17" t="str">
-        <f>IF($F8="","",I8-J8)</f>
+        <f>IF($F8="","",L8-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F8)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5311,7 +5311,7 @@
         <v/>
       </c>
       <c r="O9" s="17" t="str">
-        <f>IF($F9="","",I9-J9)</f>
+        <f>IF($F9="","",L9-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F9)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
         <v/>
       </c>
       <c r="O10" s="17" t="str">
-        <f>IF($F10="","",I10-J10)</f>
+        <f>IF($F10="","",L10-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F10)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
         <v/>
       </c>
       <c r="O11" s="17" t="str">
-        <f>IF($F11="","",I11-J11)</f>
+        <f>IF($F11="","",L11-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F11)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5482,7 +5482,7 @@
         <v/>
       </c>
       <c r="O12" s="17" t="str">
-        <f>IF($F12="","",I12-J12)</f>
+        <f>IF($F12="","",L12-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F12)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5539,7 +5539,7 @@
         <v/>
       </c>
       <c r="O13" s="17" t="str">
-        <f>IF($F13="","",I13-J13)</f>
+        <f>IF($F13="","",L13-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F13)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
         <v/>
       </c>
       <c r="O14" s="17" t="str">
-        <f>IF($F14="","",I14-J14)</f>
+        <f>IF($F14="","",L14-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F14)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5653,7 +5653,7 @@
         <v/>
       </c>
       <c r="O15" s="17" t="str">
-        <f>IF($F15="","",I15-J15)</f>
+        <f>IF($F15="","",L15-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F15)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5710,7 +5710,7 @@
         <v/>
       </c>
       <c r="O16" s="17" t="str">
-        <f>IF($F16="","",I16-J16)</f>
+        <f>IF($F16="","",L16-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F16)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5769,7 +5769,7 @@
         <v/>
       </c>
       <c r="O17" s="17" t="str">
-        <f>IF($F17="","",I17-J17)</f>
+        <f>IF($F17="","",L17-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F17)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5811,7 +5811,7 @@
         <v/>
       </c>
       <c r="O18" s="17" t="str">
-        <f>IF($F18="","",I18-J18)</f>
+        <f>IF($F18="","",L18-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F18)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5858,7 +5858,7 @@
         <v/>
       </c>
       <c r="O19" s="17" t="str">
-        <f>IF($F19="","",I19-J19)</f>
+        <f>IF($F19="","",L19-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F19)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5909,7 +5909,7 @@
         <v/>
       </c>
       <c r="O20" s="17" t="str">
-        <f>IF($F20="","",I20-J20)</f>
+        <f>IF($F20="","",L20-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F20)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
         <v/>
       </c>
       <c r="O21" s="17" t="str">
-        <f>IF($F21="","",I21-J21)</f>
+        <f>IF($F21="","",L21-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F21)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -6011,7 +6011,7 @@
         <v/>
       </c>
       <c r="O22" s="17" t="str">
-        <f>IF($F22="","",I22-J22)</f>
+        <f>IF($F22="","",L22-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F22)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -6053,7 +6053,7 @@
         <v/>
       </c>
       <c r="O23" s="17" t="str">
-        <f>IF($F23="","",I23-J23)</f>
+        <f>IF($F23="","",L23-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F23)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>
@@ -6095,7 +6095,7 @@
         <v/>
       </c>
       <c r="O24" s="17" t="str">
-        <f>IF($F24="","",I24-J24)</f>
+        <f>IF($F24="","",L24-SUMPRODUCT(('Forecast Log'!$A$5:$A$64=$F24)*('Forecast Log'!$G$5:$G$64="")*'Forecast Log'!$D$5:$D$64))</f>
         <v/>
       </c>
     </row>

</xml_diff>